<commit_message>
Json do mundo correto Parnaiba3
</commit_message>
<xml_diff>
--- a/Gazebo/todos_pontos_gps.xlsx
+++ b/Gazebo/todos_pontos_gps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K524"/>
+  <dimension ref="A1:K519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22590,7 +22590,7 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>talude_echo_fox_1</t>
+          <t>Talude1</t>
         </is>
       </c>
       <c r="B516" t="n">
@@ -22604,36 +22604,36 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>[(-3.124467165547735, -41.765491029148244), (-3.1220881755477348, -41.765429115148244)]</t>
+          <t>[(-3.125645920547735, -41.76551558214825), (-3.120909420547735, -41.76540456214824)]</t>
         </is>
       </c>
       <c r="F516" t="inlineStr">
         <is>
-          <t>[(-3.124467165547735, -41.765491029148244), (-3.1220881755477348, -41.765429115148244)]</t>
+          <t>[(-3.125645920547735, -41.76551558214825), (-3.120909420547735, -41.76540456214824)]</t>
         </is>
       </c>
       <c r="G516" t="n">
-        <v>-30.659525</v>
+        <v>-30.68701145172119</v>
       </c>
       <c r="H516" t="n">
-        <v>0.6982500000000016</v>
+        <v>0.0792705078125024</v>
       </c>
       <c r="I516" t="n">
-        <v>237.899</v>
+        <v>236.825</v>
       </c>
       <c r="J516" t="n">
-        <v>6.191400000000002</v>
+        <v>5.551000000000002</v>
       </c>
       <c r="K516" t="inlineStr">
         <is>
-          <t>ef_talude_echo_fox_1</t>
+          <t>ef_talude1</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>talude_echo_fox_2</t>
+          <t>talude2</t>
         </is>
       </c>
       <c r="B517" t="n">
@@ -22647,36 +22647,36 @@
       </c>
       <c r="E517" t="inlineStr">
         <is>
-          <t>[(-3.123286165547735, -41.76548806314825), (-3.123269175547735, -41.76543208114824)]</t>
+          <t>[(-3.123322196547735, -41.76609214114824), (-3.123233144547735, -41.764828003148246)]</t>
         </is>
       </c>
       <c r="F517" t="inlineStr">
         <is>
-          <t>[(-3.123286165547735, -41.76548806314825), (-3.123269175547735, -41.76543208114824)]</t>
+          <t>[(-3.123322196547735, -41.76609214114824), (-3.123233144547735, -41.764828003148246)]</t>
         </is>
       </c>
       <c r="G517" t="n">
-        <v>-26.15615</v>
+        <v>-64.60705</v>
       </c>
       <c r="H517" t="n">
-        <v>118.9445</v>
+        <v>-72.6447</v>
       </c>
       <c r="I517" t="n">
-        <v>1.698999999999998</v>
+        <v>4.452600000000004</v>
       </c>
       <c r="J517" t="n">
-        <v>5.5982</v>
+        <v>63.2069</v>
       </c>
       <c r="K517" t="inlineStr">
         <is>
-          <t>ef_talude_echo_fox_2</t>
+          <t>ef_talude2</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>talude_echo_fox_3</t>
+          <t>talude3</t>
         </is>
       </c>
       <c r="B518" t="n">
@@ -22690,36 +22690,36 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>[(-3.123284140547735, -41.76547737014825), (-3.1232712005477348, -41.76544277414824)]</t>
+          <t>[(-3.124991187547735, -41.76551893314824), (-3.1215641535477348, -41.765401211148244)]</t>
         </is>
       </c>
       <c r="F518" t="inlineStr">
         <is>
-          <t>[(-3.123284140547735, -41.76547737014825), (-3.1232712005477348, -41.76544277414824)]</t>
+          <t>[(-3.124991187547735, -41.76551893314824), (-3.1215641535477348, -41.765401211148244)]</t>
         </is>
       </c>
       <c r="G518" t="n">
-        <v>-17.577575</v>
+        <v>77.8729</v>
       </c>
       <c r="H518" t="n">
-        <v>118.88475</v>
+        <v>13.937325</v>
       </c>
       <c r="I518" t="n">
-        <v>1.293999999999997</v>
+        <v>171.3517</v>
       </c>
       <c r="J518" t="n">
-        <v>3.459599999999998</v>
+        <v>5.886099999999999</v>
       </c>
       <c r="K518" t="inlineStr">
         <is>
-          <t>ef_talude_echo_fox_3</t>
+          <t>ef_talude3</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>talude_fox</t>
+          <t>talude4</t>
         </is>
       </c>
       <c r="B519" t="n">
@@ -22733,244 +22733,29 @@
       </c>
       <c r="E519" t="inlineStr">
         <is>
-          <t>[(-3.123302022547735, -41.76577286264824), (-3.123253318547735, -41.76514728164825)]</t>
+          <t>[(-3.123325899547735, -41.765905913148245), (-3.123229441547735, -41.76501423114824)]</t>
         </is>
       </c>
       <c r="F519" t="inlineStr">
         <is>
-          <t>[(-3.123302022547735, -41.76577286264824), (-3.123253318547735, -41.76514728164825)]</t>
+          <t>[(-3.123325899547735, -41.765905913148245), (-3.123229441547735, -41.76501423114824)]</t>
         </is>
       </c>
       <c r="G519" t="n">
-        <v>-64.687775</v>
+        <v>96.6101</v>
       </c>
       <c r="H519" t="n">
-        <v>-72.78302500000001</v>
+        <v>-74.260575</v>
       </c>
       <c r="I519" t="n">
-        <v>4.87039999999999</v>
+        <v>4.822900000000004</v>
       </c>
       <c r="J519" t="n">
-        <v>62.5581</v>
+        <v>44.58409999999999</v>
       </c>
       <c r="K519" t="inlineStr">
         <is>
-          <t>ef_talude_fox</t>
-        </is>
-      </c>
-    </row>
-    <row r="520">
-      <c r="A520" t="inlineStr">
-        <is>
-          <t>talude_echo_fox_5</t>
-        </is>
-      </c>
-      <c r="B520" t="n">
-        <v>-3.123277670547735</v>
-      </c>
-      <c r="C520" t="n">
-        <v>-41.76546007214824</v>
-      </c>
-      <c r="D520" t="n">
-        <v>77</v>
-      </c>
-      <c r="E520" t="inlineStr">
-        <is>
-          <t>[(-3.123407665547735, -41.765484589648246), (-3.123147675547735, -41.76543555464824)]</t>
-        </is>
-      </c>
-      <c r="F520" t="inlineStr">
-        <is>
-          <t>[(-3.123407665547735, -41.765484589648246), (-3.123147675547735, -41.76543555464824)]</t>
-        </is>
-      </c>
-      <c r="G520" t="n">
-        <v>-32.317</v>
-      </c>
-      <c r="H520" t="n">
-        <v>-141.65625</v>
-      </c>
-      <c r="I520" t="n">
-        <v>25.999</v>
-      </c>
-      <c r="J520" t="n">
-        <v>4.903499999999998</v>
-      </c>
-      <c r="K520" t="inlineStr">
-        <is>
-          <t>ef_talude_echo_fox_5</t>
-        </is>
-      </c>
-    </row>
-    <row r="521">
-      <c r="A521" t="inlineStr">
-        <is>
-          <t>talude_bravo</t>
-        </is>
-      </c>
-      <c r="B521" t="n">
-        <v>-3.123277670547735</v>
-      </c>
-      <c r="C521" t="n">
-        <v>-41.76546007214824</v>
-      </c>
-      <c r="D521" t="n">
-        <v>77</v>
-      </c>
-      <c r="E521" t="inlineStr">
-        <is>
-          <t>[(-3.123339318047735, -41.76547506214824), (-3.123216023047735, -41.76544508214825)]</t>
-        </is>
-      </c>
-      <c r="F521" t="inlineStr">
-        <is>
-          <t>[(-3.123339318047735, -41.76547506214824), (-3.123216023047735, -41.76544508214825)]</t>
-        </is>
-      </c>
-      <c r="G521" t="n">
-        <v>125.2925</v>
-      </c>
-      <c r="H521" t="n">
-        <v>-70.693375</v>
-      </c>
-      <c r="I521" t="n">
-        <v>12.32950000000001</v>
-      </c>
-      <c r="J521" t="n">
-        <v>2.99799999999999</v>
-      </c>
-      <c r="K521" t="inlineStr">
-        <is>
-          <t>ef_talude_bravo</t>
-        </is>
-      </c>
-    </row>
-    <row r="522">
-      <c r="A522" t="inlineStr">
-        <is>
-          <t>talude_bravo_2</t>
-        </is>
-      </c>
-      <c r="B522" t="n">
-        <v>-3.123277670547735</v>
-      </c>
-      <c r="C522" t="n">
-        <v>-41.76546007214824</v>
-      </c>
-      <c r="D522" t="n">
-        <v>77</v>
-      </c>
-      <c r="E522" t="inlineStr">
-        <is>
-          <t>[(-3.123301995547735, -41.765651081648244), (-3.123253345547735, -41.765269062648244)]</t>
-        </is>
-      </c>
-      <c r="F522" t="inlineStr">
-        <is>
-          <t>[(-3.123301995547735, -41.765651081648244), (-3.123253345547735, -41.765269062648244)]</t>
-        </is>
-      </c>
-      <c r="G522" t="n">
-        <v>99.41840000000001</v>
-      </c>
-      <c r="H522" t="n">
-        <v>-74.3254</v>
-      </c>
-      <c r="I522" t="n">
-        <v>4.86500000000001</v>
-      </c>
-      <c r="J522" t="n">
-        <v>38.2019</v>
-      </c>
-      <c r="K522" t="inlineStr">
-        <is>
-          <t>ef_talude_bravo_2</t>
-        </is>
-      </c>
-    </row>
-    <row r="523">
-      <c r="A523" t="inlineStr">
-        <is>
-          <t>talude_bravo_3</t>
-        </is>
-      </c>
-      <c r="B523" t="n">
-        <v>-3.123277670547735</v>
-      </c>
-      <c r="C523" t="n">
-        <v>-41.76546007214824</v>
-      </c>
-      <c r="D523" t="n">
-        <v>77</v>
-      </c>
-      <c r="E523" t="inlineStr">
-        <is>
-          <t>[(-3.124158346047735, -41.76549137214825), (-3.122396995047735, -41.76542877214824)]</t>
-        </is>
-      </c>
-      <c r="F523" t="inlineStr">
-        <is>
-          <t>[(-3.124158346047735, -41.76549137214825), (-3.122396995047735, -41.76542877214824)]</t>
-        </is>
-      </c>
-      <c r="G523" t="n">
-        <v>77.84765000000002</v>
-      </c>
-      <c r="H523" t="n">
-        <v>11.411375</v>
-      </c>
-      <c r="I523" t="n">
-        <v>176.1351</v>
-      </c>
-      <c r="J523" t="n">
-        <v>6.260000000000006</v>
-      </c>
-      <c r="K523" t="inlineStr">
-        <is>
-          <t>ef_talude_bravo_3</t>
-        </is>
-      </c>
-    </row>
-    <row r="524">
-      <c r="A524" t="inlineStr">
-        <is>
-          <t>talude_echo_fox1</t>
-        </is>
-      </c>
-      <c r="B524" t="n">
-        <v>-3.123277670547735</v>
-      </c>
-      <c r="C524" t="n">
-        <v>-41.76546007214824</v>
-      </c>
-      <c r="D524" t="n">
-        <v>77</v>
-      </c>
-      <c r="E524" t="inlineStr">
-        <is>
-          <t>[(-3.125652900547735, -41.76550457714824), (-3.120902440547735, -41.765415567148246)]</t>
-        </is>
-      </c>
-      <c r="F524" t="inlineStr">
-        <is>
-          <t>[(-3.125652900547735, -41.76550457714824), (-3.120902440547735, -41.765415567148246)]</t>
-        </is>
-      </c>
-      <c r="G524" t="n">
-        <v>-31.358175</v>
-      </c>
-      <c r="H524" t="n">
-        <v>0.7434999999999974</v>
-      </c>
-      <c r="I524" t="n">
-        <v>237.523</v>
-      </c>
-      <c r="J524" t="n">
-        <v>4.450500000000002</v>
-      </c>
-      <c r="K524" t="inlineStr">
-        <is>
-          <t>ef_talude_echo_fox1</t>
+          <t>ef_talude4</t>
         </is>
       </c>
     </row>

</xml_diff>